<commit_message>
Add new assets, SVG logos, HTML pages, and update index with latest features
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assests/AmpTest claud4.xlsx
+++ b/assests/AmpTest claud4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/toddanderson/Documents/claude projects/amplifinder/assests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1143CEE-83BF-FB4D-819E-B2F63B70EBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55C39E4-6EFF-934F-968E-A9EA534DC8EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="740" yWindow="660" windowWidth="27640" windowHeight="16760" xr2:uid="{A2AA72AD-F933-604F-82A4-82C55EAB3989}"/>
   </bookViews>
@@ -167,9 +167,6 @@
     <t xml:space="preserve">Performance </t>
   </si>
   <si>
-    <t xml:space="preserve">Coverage </t>
-  </si>
-  <si>
     <t xml:space="preserve">MOS SUB </t>
   </si>
   <si>
@@ -197,9 +194,6 @@
     <t>AMD210</t>
   </si>
   <si>
-    <t>Coverage</t>
-  </si>
-  <si>
     <t>10HDR</t>
   </si>
   <si>
@@ -225,6 +219,12 @@
   </si>
   <si>
     <t>DSUB6F5K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enhancement </t>
+  </si>
+  <si>
+    <t>Enhancement</t>
   </si>
 </sst>
 </file>
@@ -689,13 +689,13 @@
         <v>250.1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>42</v>
@@ -721,10 +721,10 @@
         <v>250.2</v>
       </c>
       <c r="G3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" t="s">
         <v>44</v>
-      </c>
-      <c r="J3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -760,10 +760,10 @@
         <v>250.4</v>
       </c>
       <c r="G5" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" t="s">
         <v>44</v>
-      </c>
-      <c r="J5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -782,10 +782,10 @@
         <v>250.4</v>
       </c>
       <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
         <v>44</v>
-      </c>
-      <c r="J6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -821,10 +821,10 @@
         <v>250.4</v>
       </c>
       <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" t="s">
         <v>44</v>
-      </c>
-      <c r="J8" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -843,10 +843,10 @@
         <v>250.4</v>
       </c>
       <c r="G9" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" t="s">
         <v>44</v>
-      </c>
-      <c r="J9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -880,10 +880,10 @@
         <v>8</v>
       </c>
       <c r="G11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" t="s">
         <v>44</v>
-      </c>
-      <c r="J11" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -900,10 +900,10 @@
         <v>9</v>
       </c>
       <c r="G12" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" t="s">
         <v>44</v>
-      </c>
-      <c r="J12" t="s">
-        <v>45</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -941,10 +941,10 @@
         <v>250.2</v>
       </c>
       <c r="G14" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" t="s">
         <v>46</v>
-      </c>
-      <c r="J14" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -976,10 +976,10 @@
         <v>250.4</v>
       </c>
       <c r="G16" t="s">
+        <v>45</v>
+      </c>
+      <c r="J16" t="s">
         <v>46</v>
-      </c>
-      <c r="J16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.2">
@@ -996,10 +996,10 @@
         <v>250.4</v>
       </c>
       <c r="G17" t="s">
+        <v>45</v>
+      </c>
+      <c r="J17" t="s">
         <v>46</v>
-      </c>
-      <c r="J17" t="s">
-        <v>47</v>
       </c>
       <c r="L17" s="1"/>
     </row>
@@ -1032,10 +1032,10 @@
         <v>250.4</v>
       </c>
       <c r="G19" t="s">
+        <v>45</v>
+      </c>
+      <c r="J19" t="s">
         <v>46</v>
-      </c>
-      <c r="J19" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
@@ -1052,10 +1052,10 @@
         <v>250.4</v>
       </c>
       <c r="G20" t="s">
+        <v>45</v>
+      </c>
+      <c r="J20" t="s">
         <v>46</v>
-      </c>
-      <c r="J20" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
@@ -1087,10 +1087,10 @@
         <v>11</v>
       </c>
       <c r="G22" t="s">
+        <v>45</v>
+      </c>
+      <c r="J22" t="s">
         <v>46</v>
-      </c>
-      <c r="J22" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.2">
@@ -1107,10 +1107,10 @@
         <v>12</v>
       </c>
       <c r="G23" t="s">
+        <v>45</v>
+      </c>
+      <c r="J23" t="s">
         <v>46</v>
-      </c>
-      <c r="J23" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.2">
@@ -1146,10 +1146,10 @@
         <v>250.2</v>
       </c>
       <c r="G25" t="s">
+        <v>45</v>
+      </c>
+      <c r="J25" t="s">
         <v>46</v>
-      </c>
-      <c r="J25" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
@@ -1181,10 +1181,10 @@
         <v>250.4</v>
       </c>
       <c r="G27" t="s">
+        <v>45</v>
+      </c>
+      <c r="J27" t="s">
         <v>46</v>
-      </c>
-      <c r="J27" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.2">
@@ -1201,10 +1201,10 @@
         <v>250.4</v>
       </c>
       <c r="G28" t="s">
+        <v>45</v>
+      </c>
+      <c r="J28" t="s">
         <v>46</v>
-      </c>
-      <c r="J28" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
@@ -1236,10 +1236,10 @@
         <v>250.4</v>
       </c>
       <c r="G30" t="s">
+        <v>45</v>
+      </c>
+      <c r="J30" t="s">
         <v>46</v>
-      </c>
-      <c r="J30" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.2">
@@ -1256,10 +1256,10 @@
         <v>250.4</v>
       </c>
       <c r="G31" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" t="s">
         <v>46</v>
-      </c>
-      <c r="J31" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.2">
@@ -1291,10 +1291,10 @@
         <v>8</v>
       </c>
       <c r="G33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J33" t="s">
         <v>46</v>
-      </c>
-      <c r="J33" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -1311,10 +1311,10 @@
         <v>9</v>
       </c>
       <c r="G34" t="s">
+        <v>45</v>
+      </c>
+      <c r="J34" t="s">
         <v>46</v>
-      </c>
-      <c r="J34" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
@@ -1350,10 +1350,10 @@
         <v>250.2</v>
       </c>
       <c r="G36" t="s">
+        <v>45</v>
+      </c>
+      <c r="J36" t="s">
         <v>46</v>
-      </c>
-      <c r="J36" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -1386,10 +1386,10 @@
         <v>250.4</v>
       </c>
       <c r="G38" t="s">
+        <v>45</v>
+      </c>
+      <c r="J38" t="s">
         <v>46</v>
-      </c>
-      <c r="J38" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -1406,10 +1406,10 @@
         <v>250.4</v>
       </c>
       <c r="G39" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" t="s">
         <v>46</v>
-      </c>
-      <c r="J39" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1442,10 +1442,10 @@
         <v>250.4</v>
       </c>
       <c r="G41" t="s">
+        <v>45</v>
+      </c>
+      <c r="J41" t="s">
         <v>46</v>
-      </c>
-      <c r="J41" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
@@ -1462,10 +1462,10 @@
         <v>250.4</v>
       </c>
       <c r="G42" t="s">
+        <v>45</v>
+      </c>
+      <c r="J42" t="s">
         <v>46</v>
-      </c>
-      <c r="J42" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
@@ -1498,10 +1498,10 @@
         <v>8</v>
       </c>
       <c r="G44" t="s">
+        <v>45</v>
+      </c>
+      <c r="J44" t="s">
         <v>46</v>
-      </c>
-      <c r="J44" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -1518,10 +1518,10 @@
         <v>9</v>
       </c>
       <c r="G45" t="s">
+        <v>45</v>
+      </c>
+      <c r="J45" t="s">
         <v>46</v>
-      </c>
-      <c r="J45" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -1573,19 +1573,19 @@
         <v>250.1</v>
       </c>
       <c r="G48" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I48" t="s">
         <v>54</v>
       </c>
-      <c r="H48" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I48" t="s">
+      <c r="J48" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K48" t="s">
         <v>56</v>
-      </c>
-      <c r="J48" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K48" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.2">
@@ -1602,16 +1602,16 @@
         <v>1000.2</v>
       </c>
       <c r="G49" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I49" t="s">
         <v>54</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K49" t="s">
         <v>56</v>
-      </c>
-      <c r="J49" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K49" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.2">
@@ -1656,19 +1656,19 @@
         <v>1000.4</v>
       </c>
       <c r="G52" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I52" t="s">
         <v>54</v>
       </c>
-      <c r="H52" s="1" t="s">
+      <c r="J52" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I52" t="s">
+      <c r="K52" t="s">
         <v>56</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K52" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.2">
@@ -1685,19 +1685,19 @@
         <v>1000.4</v>
       </c>
       <c r="G53" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I53" t="s">
         <v>54</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I53" t="s">
+      <c r="K53" t="s">
         <v>56</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K53" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.2">
@@ -1714,19 +1714,19 @@
         <v>1000.4</v>
       </c>
       <c r="G54" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I54" t="s">
         <v>54</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I54" t="s">
+      <c r="K54" t="s">
         <v>56</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K54" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.2">
@@ -1743,19 +1743,19 @@
         <v>1000.4</v>
       </c>
       <c r="G55" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I55" t="s">
         <v>54</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I55" t="s">
+      <c r="K55" t="s">
         <v>56</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K55" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.2">
@@ -1803,19 +1803,19 @@
         <v>250.1</v>
       </c>
       <c r="G58" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I58" t="s">
         <v>54</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I58" t="s">
+      <c r="K58" t="s">
         <v>56</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K58" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.2">
@@ -1832,19 +1832,19 @@
         <v>1000.2</v>
       </c>
       <c r="G59" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I59" t="s">
         <v>54</v>
       </c>
-      <c r="H59" s="1" t="s">
+      <c r="J59" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I59" t="s">
+      <c r="K59" t="s">
         <v>56</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K59" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.2">
@@ -1872,7 +1872,7 @@
         <v>0</v>
       </c>
       <c r="F61" s="1">
-        <v>1000.2</v>
+        <v>250.2</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.2">
@@ -1889,19 +1889,19 @@
         <v>1000.4</v>
       </c>
       <c r="G62" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I62" t="s">
         <v>54</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I62" t="s">
+      <c r="K62" t="s">
         <v>56</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K62" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.2">
@@ -1918,19 +1918,19 @@
         <v>1000.4</v>
       </c>
       <c r="G63" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I63" t="s">
         <v>54</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I63" t="s">
+      <c r="K63" t="s">
         <v>56</v>
-      </c>
-      <c r="J63" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K63" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.2">
@@ -1947,19 +1947,19 @@
         <v>1000.4</v>
       </c>
       <c r="G64" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I64" t="s">
         <v>54</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I64" t="s">
+      <c r="K64" t="s">
         <v>56</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K64" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.2">
@@ -1976,19 +1976,19 @@
         <v>1000.4</v>
       </c>
       <c r="G65" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I65" t="s">
         <v>54</v>
       </c>
-      <c r="H65" s="1" t="s">
+      <c r="J65" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I65" t="s">
+      <c r="K65" t="s">
         <v>56</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K65" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.2">
@@ -2036,19 +2036,19 @@
         <v>250.1</v>
       </c>
       <c r="G68" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I68" t="s">
         <v>54</v>
       </c>
-      <c r="H68" s="1" t="s">
+      <c r="J68" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I68" t="s">
+      <c r="K68" t="s">
         <v>56</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K68" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.2">
@@ -2065,19 +2065,19 @@
         <v>1000.2</v>
       </c>
       <c r="G69" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I69" t="s">
         <v>54</v>
       </c>
-      <c r="H69" s="1" t="s">
+      <c r="J69" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I69" t="s">
+      <c r="K69" t="s">
         <v>56</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K69" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.2">
@@ -2122,19 +2122,19 @@
         <v>1000.4</v>
       </c>
       <c r="G72" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I72" t="s">
         <v>54</v>
       </c>
-      <c r="H72" s="1" t="s">
+      <c r="J72" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I72" t="s">
+      <c r="K72" t="s">
         <v>56</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K72" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.2">
@@ -2151,19 +2151,19 @@
         <v>1000.4</v>
       </c>
       <c r="G73" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I73" t="s">
         <v>54</v>
       </c>
-      <c r="H73" s="1" t="s">
+      <c r="J73" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I73" t="s">
+      <c r="K73" t="s">
         <v>56</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K73" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.2">
@@ -2180,19 +2180,19 @@
         <v>1000.4</v>
       </c>
       <c r="G74" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I74" t="s">
         <v>54</v>
       </c>
-      <c r="H74" s="1" t="s">
+      <c r="J74" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I74" t="s">
+      <c r="K74" t="s">
         <v>56</v>
-      </c>
-      <c r="J74" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K74" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.2">
@@ -2209,19 +2209,19 @@
         <v>1000.4</v>
       </c>
       <c r="G75" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I75" t="s">
         <v>54</v>
       </c>
-      <c r="H75" s="1" t="s">
+      <c r="J75" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I75" t="s">
+      <c r="K75" t="s">
         <v>56</v>
-      </c>
-      <c r="J75" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K75" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.2">
@@ -2559,16 +2559,16 @@
         <v>250.1</v>
       </c>
       <c r="G98" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H98" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K98" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="99" spans="2:11" x14ac:dyDescent="0.2">
@@ -2585,16 +2585,16 @@
         <v>1000.2</v>
       </c>
       <c r="G99" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H99" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K99" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.2">
@@ -2641,16 +2641,16 @@
         <v>1000.4</v>
       </c>
       <c r="G102" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H102" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K102" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="103" spans="2:11" x14ac:dyDescent="0.2">
@@ -2667,16 +2667,16 @@
         <v>1000.4</v>
       </c>
       <c r="G103" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H103" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J103" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K103" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="104" spans="2:11" x14ac:dyDescent="0.2">
@@ -2693,16 +2693,16 @@
         <v>1000.4</v>
       </c>
       <c r="G104" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H104" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K104" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.2">
@@ -2767,16 +2767,16 @@
         <v>250.1</v>
       </c>
       <c r="G108" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H108" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J108" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K108" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="109" spans="2:11" x14ac:dyDescent="0.2">
@@ -2793,16 +2793,16 @@
         <v>1000.2</v>
       </c>
       <c r="G109" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H109" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J109" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K109" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="110" spans="2:11" x14ac:dyDescent="0.2">
@@ -2849,16 +2849,16 @@
         <v>1000.4</v>
       </c>
       <c r="G112" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H112" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J112" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K112" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
@@ -2875,16 +2875,16 @@
         <v>1000.4</v>
       </c>
       <c r="G113" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H113" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J113" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K113" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.2">
@@ -2901,16 +2901,16 @@
         <v>1000.4</v>
       </c>
       <c r="G114" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H114" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J114" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K114" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.2">
@@ -2927,16 +2927,16 @@
         <v>1000.4</v>
       </c>
       <c r="G115" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H115" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J115" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K115" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.2">
@@ -2971,16 +2971,16 @@
         <v>250.2</v>
       </c>
       <c r="G117" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H117" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J117" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K117" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.2">
@@ -2997,16 +2997,16 @@
         <v>250.4</v>
       </c>
       <c r="G118" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H118" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J118" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K118" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.2">
@@ -3038,16 +3038,16 @@
         <v>250.4</v>
       </c>
       <c r="G120" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H120" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J120" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K120" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.2">
@@ -3064,16 +3064,16 @@
         <v>250.4</v>
       </c>
       <c r="G121" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H121" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J121" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K121" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.2">
@@ -3141,7 +3141,7 @@
         <v>250.2</v>
       </c>
       <c r="G125" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.2">
@@ -3158,7 +3158,7 @@
         <v>250.4</v>
       </c>
       <c r="G126" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.2">
@@ -3175,7 +3175,7 @@
         <v>250.4</v>
       </c>
       <c r="G127" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.2">
@@ -3240,7 +3240,7 @@
         <v>250.2</v>
       </c>
       <c r="G131" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="132" spans="2:11" x14ac:dyDescent="0.2">
@@ -3257,7 +3257,7 @@
         <v>250.4</v>
       </c>
       <c r="G132" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="133" spans="2:11" x14ac:dyDescent="0.2">
@@ -3274,7 +3274,7 @@
         <v>250.4</v>
       </c>
       <c r="G133" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="134" spans="2:11" x14ac:dyDescent="0.2">
@@ -3339,7 +3339,7 @@
         <v>250.1</v>
       </c>
       <c r="G137" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="138" spans="2:11" x14ac:dyDescent="0.2">
@@ -3356,7 +3356,7 @@
         <v>250.2</v>
       </c>
       <c r="G138" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="139" spans="2:11" x14ac:dyDescent="0.2">
@@ -3373,7 +3373,7 @@
         <v>250.4</v>
       </c>
       <c r="G139" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="140" spans="2:11" x14ac:dyDescent="0.2">
@@ -3438,10 +3438,10 @@
         <v>1000.2</v>
       </c>
       <c r="G143" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J143" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="144" spans="2:11" x14ac:dyDescent="0.2">
@@ -3458,10 +3458,10 @@
         <v>1000.4</v>
       </c>
       <c r="G144" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J144" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K144" s="1"/>
     </row>
@@ -3479,10 +3479,10 @@
         <v>1000.2</v>
       </c>
       <c r="G145" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J145" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K145" s="1"/>
     </row>
@@ -3580,7 +3580,7 @@
         <v>1000.2</v>
       </c>
       <c r="G151" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.2">
@@ -3597,7 +3597,7 @@
         <v>1000.4</v>
       </c>
       <c r="G152" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I152" s="1"/>
       <c r="J152" s="1"/>
@@ -3617,7 +3617,7 @@
         <v>1000.4</v>
       </c>
       <c r="G153" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I153" s="1"/>
       <c r="J153" s="1"/>
@@ -3636,7 +3636,7 @@
         <v>38</v>
       </c>
       <c r="G154" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I154" s="1"/>
       <c r="J154" s="1"/>
@@ -3655,7 +3655,7 @@
         <v>39</v>
       </c>
       <c r="G155" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I155" s="1"/>
       <c r="J155" s="1"/>
@@ -3674,7 +3674,7 @@
         <v>1000.4</v>
       </c>
       <c r="G156" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I156" s="1"/>
       <c r="J156" s="1"/>
@@ -3693,7 +3693,7 @@
         <v>1000.4</v>
       </c>
       <c r="G157" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I157" s="1"/>
       <c r="J157" s="1"/>
@@ -3712,7 +3712,7 @@
         <v>1000.4</v>
       </c>
       <c r="G158" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I158" s="1"/>
       <c r="J158" s="1"/>
@@ -3731,7 +3731,7 @@
         <v>38</v>
       </c>
       <c r="G159" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I159" s="1"/>
       <c r="J159" s="1"/>
@@ -3750,7 +3750,7 @@
         <v>39</v>
       </c>
       <c r="G160" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I160" s="1"/>
       <c r="J160" s="1"/>
@@ -3844,7 +3844,7 @@
         <v>1000.1</v>
       </c>
       <c r="G166" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.2">
@@ -3861,7 +3861,7 @@
         <v>1000.2</v>
       </c>
       <c r="G167" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I167" s="1"/>
       <c r="J167" s="1"/>
@@ -3880,7 +3880,7 @@
         <v>1000.2</v>
       </c>
       <c r="G168" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I168" s="1"/>
       <c r="J168" s="1"/>
@@ -3899,7 +3899,7 @@
         <v>1000.4</v>
       </c>
       <c r="G169" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I169" s="1"/>
       <c r="J169" s="1"/>
@@ -3918,7 +3918,7 @@
         <v>1000.4</v>
       </c>
       <c r="G170" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I170" s="1"/>
       <c r="J170" s="1"/>
@@ -3937,7 +3937,7 @@
         <v>1000.2</v>
       </c>
       <c r="G171" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I171" s="1"/>
       <c r="J171" s="1"/>
@@ -3956,7 +3956,7 @@
         <v>1000.2</v>
       </c>
       <c r="G172" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I172" s="1"/>
       <c r="J172" s="1"/>
@@ -3975,7 +3975,7 @@
         <v>1000.4</v>
       </c>
       <c r="G173" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I173" s="1"/>
       <c r="J173" s="1"/>
@@ -3994,7 +3994,7 @@
         <v>1000.4</v>
       </c>
       <c r="G174" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I174" s="1"/>
       <c r="J174" s="1"/>
@@ -4013,7 +4013,7 @@
         <v>1000.4</v>
       </c>
       <c r="G175" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I175" s="1"/>
       <c r="J175" s="1"/>
@@ -4023,7 +4023,7 @@
         <v>41</v>
       </c>
       <c r="B176" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>21</v>
@@ -4054,13 +4054,13 @@
         <v>250.2</v>
       </c>
       <c r="G177" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H177" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I177" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="178" spans="2:9" x14ac:dyDescent="0.2">
@@ -4091,13 +4091,13 @@
         <v>250.4</v>
       </c>
       <c r="G179" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H179" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I179" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="180" spans="2:9" x14ac:dyDescent="0.2">
@@ -4114,13 +4114,13 @@
         <v>250.4</v>
       </c>
       <c r="G180" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H180" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I180" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="181" spans="2:9" x14ac:dyDescent="0.2">
@@ -4151,13 +4151,13 @@
         <v>250.4</v>
       </c>
       <c r="G182" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H182" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I182" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="183" spans="2:9" x14ac:dyDescent="0.2">
@@ -4174,13 +4174,13 @@
         <v>250.4</v>
       </c>
       <c r="G183" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H183" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I183" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="184" spans="2:9" x14ac:dyDescent="0.2">
@@ -4211,13 +4211,13 @@
         <v>11</v>
       </c>
       <c r="G185" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H185" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I185" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="186" spans="2:9" x14ac:dyDescent="0.2">
@@ -4234,18 +4234,18 @@
         <v>12</v>
       </c>
       <c r="G186" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H186" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I186" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="187" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B187" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>21</v>
@@ -4274,13 +4274,13 @@
         <v>250.2</v>
       </c>
       <c r="G188" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H188" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I188" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="189" spans="2:9" x14ac:dyDescent="0.2">
@@ -4311,13 +4311,13 @@
         <v>250.4</v>
       </c>
       <c r="G190" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H190" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I190" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="191" spans="2:9" x14ac:dyDescent="0.2">
@@ -4334,13 +4334,13 @@
         <v>250.4</v>
       </c>
       <c r="G191" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H191" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I191" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="192" spans="2:9" x14ac:dyDescent="0.2">
@@ -4371,13 +4371,13 @@
         <v>250.4</v>
       </c>
       <c r="G193" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H193" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I193" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="194" spans="2:9" x14ac:dyDescent="0.2">
@@ -4394,13 +4394,13 @@
         <v>250.4</v>
       </c>
       <c r="G194" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I194" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="195" spans="2:9" x14ac:dyDescent="0.2">
@@ -4431,13 +4431,13 @@
         <v>8</v>
       </c>
       <c r="G196" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H196" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I196" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="197" spans="2:9" x14ac:dyDescent="0.2">
@@ -4454,18 +4454,18 @@
         <v>9</v>
       </c>
       <c r="G197" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H197" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I197" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="198" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B198" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>21</v>
@@ -4494,13 +4494,13 @@
         <v>250.2</v>
       </c>
       <c r="G199" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H199" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I199" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="200" spans="2:9" x14ac:dyDescent="0.2">
@@ -4531,13 +4531,13 @@
         <v>250.4</v>
       </c>
       <c r="G201" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H201" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I201" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="202" spans="2:9" x14ac:dyDescent="0.2">
@@ -4554,13 +4554,13 @@
         <v>250.4</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H202" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I202" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="203" spans="2:9" x14ac:dyDescent="0.2">
@@ -4591,13 +4591,13 @@
         <v>250.4</v>
       </c>
       <c r="G204" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H204" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I204" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="205" spans="2:9" x14ac:dyDescent="0.2">
@@ -4614,13 +4614,13 @@
         <v>250.4</v>
       </c>
       <c r="G205" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H205" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I205" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="206" spans="2:9" x14ac:dyDescent="0.2">
@@ -4651,13 +4651,13 @@
         <v>8</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H207" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I207" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="208" spans="2:9" x14ac:dyDescent="0.2">
@@ -4674,18 +4674,18 @@
         <v>9</v>
       </c>
       <c r="G208" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H208" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I208" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="209" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B209" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>21</v>
@@ -4714,13 +4714,13 @@
         <v>250.2</v>
       </c>
       <c r="G210" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H210" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I210" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="211" spans="2:9" x14ac:dyDescent="0.2">
@@ -4751,13 +4751,13 @@
         <v>250.4</v>
       </c>
       <c r="G212" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H212" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I212" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="213" spans="2:9" x14ac:dyDescent="0.2">
@@ -4774,13 +4774,13 @@
         <v>250.4</v>
       </c>
       <c r="G213" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H213" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I213" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="214" spans="2:9" x14ac:dyDescent="0.2">
@@ -4811,13 +4811,13 @@
         <v>250.4</v>
       </c>
       <c r="G215" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H215" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I215" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="216" spans="2:9" x14ac:dyDescent="0.2">
@@ -4834,13 +4834,13 @@
         <v>250.4</v>
       </c>
       <c r="G216" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H216" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I216" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="217" spans="2:9" x14ac:dyDescent="0.2">
@@ -4871,13 +4871,13 @@
         <v>8</v>
       </c>
       <c r="G218" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H218" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I218" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="219" spans="2:9" x14ac:dyDescent="0.2">
@@ -4894,13 +4894,13 @@
         <v>9</v>
       </c>
       <c r="G219" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I219" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>